<commit_message>
Inventario al 21.10.2026, correos autorizados y selector de sucursal para gerentes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014ASsM9mcqYrhrTsJC3CpHT
</commit_message>
<xml_diff>
--- a/plantillas/0.xlsx
+++ b/plantillas/0.xlsx
@@ -9485,7 +9485,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -9505,7 +9505,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -9545,7 +9545,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -9665,7 +9665,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -9945,7 +9945,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -10445,7 +10445,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -10665,7 +10665,7 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -10905,7 +10905,7 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -11185,7 +11185,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -11405,7 +11405,7 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
@@ -11443,7 +11443,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>20.10.2026</t>
+          <t>21.10.2026</t>
         </is>
       </c>
     </row>

</xml_diff>